<commit_message>
“menambahkan fitur upload gambar di buku_tamu”
</commit_message>
<xml_diff>
--- a/Laporan Buku Tamu.xlsx
+++ b/Laporan Buku Tamu.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
   <si>
     <t>No</t>
   </si>
@@ -38,70 +38,19 @@
     <t>KEPENTINGAN</t>
   </si>
   <si>
-    <t>2026-09-01</t>
-  </si>
-  <si>
-    <t>Mike</t>
-  </si>
-  <si>
-    <t>Griya Maleber</t>
-  </si>
-  <si>
-    <t>08123456789</t>
-  </si>
-  <si>
-    <t>Jax</t>
-  </si>
-  <si>
-    <t>Keperluan administrasi</t>
-  </si>
-  <si>
-    <t>2026-09-02</t>
-  </si>
-  <si>
-    <t>Miles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cianjur </t>
-  </si>
-  <si>
-    <t>085656567</t>
-  </si>
-  <si>
-    <t>guru</t>
-  </si>
-  <si>
-    <t>minjem buku</t>
-  </si>
-  <si>
-    <t>2026-09-03</t>
-  </si>
-  <si>
-    <t>iqbal</t>
-  </si>
-  <si>
-    <t>pesona</t>
-  </si>
-  <si>
-    <t>0822243455</t>
-  </si>
-  <si>
-    <t>akhdan</t>
-  </si>
-  <si>
-    <t>membaca</t>
-  </si>
-  <si>
-    <t>2026-09-14</t>
-  </si>
-  <si>
-    <t>shion</t>
-  </si>
-  <si>
-    <t>kyoto</t>
-  </si>
-  <si>
-    <t>pribadi</t>
+    <t>2026-09-23</t>
+  </si>
+  <si>
+    <t>jax</t>
+  </si>
+  <si>
+    <t>german</t>
+  </si>
+  <si>
+    <t>mike</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ngobrol </t>
   </si>
 </sst>
 </file>
@@ -441,7 +390,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -480,83 +429,14 @@
       <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2">
+        <v>1123445355</v>
+      </c>
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5">
-        <v>34342525</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>